<commit_message>
modificaciones. Tengo que realizar los análisis de Ks por cada area nueva
</commit_message>
<xml_diff>
--- a/Tabla_Nvasosnuevos.xlsx
+++ b/Tabla_Nvasosnuevos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\minicores\Qca_Bruto\Minicores-Q.canariensis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CCF7FE-F152-482F-984B-032F6411E95A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41092F9C-7644-498C-ACDE-0C9322140032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="newvess" sheetId="1" r:id="rId1"/>
@@ -30622,7 +30622,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>76000</v>
+        <v>760000</v>
       </c>
       <c r="C2" s="10">
         <v>44329</v>
@@ -30633,7 +30633,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>16000</v>
+        <v>160000</v>
       </c>
       <c r="C3" s="10">
         <v>44343</v>
@@ -30644,7 +30644,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>73000</v>
+        <v>730000</v>
       </c>
       <c r="C4" s="10">
         <v>44399</v>
@@ -30655,7 +30655,7 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <v>132000</v>
+        <v>1320000</v>
       </c>
       <c r="C5" s="10">
         <v>44448</v>
@@ -30666,7 +30666,7 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <v>274900</v>
+        <v>2749000</v>
       </c>
       <c r="C6" s="10">
         <v>44483</v>
@@ -30677,7 +30677,7 @@
         <v>2</v>
       </c>
       <c r="B7">
-        <v>20090</v>
+        <v>200900</v>
       </c>
       <c r="C7" s="10">
         <v>44546</v>
@@ -30688,7 +30688,7 @@
         <v>2</v>
       </c>
       <c r="B8">
-        <v>5640</v>
+        <v>56400</v>
       </c>
       <c r="C8" s="10">
         <v>44215</v>
@@ -30699,7 +30699,7 @@
         <v>3</v>
       </c>
       <c r="B9">
-        <v>287000</v>
+        <v>2870000</v>
       </c>
       <c r="C9" s="10">
         <v>44287</v>
@@ -30710,7 +30710,7 @@
         <v>3</v>
       </c>
       <c r="B10">
-        <v>91039</v>
+        <v>910390</v>
       </c>
       <c r="C10" s="10">
         <v>44315</v>
@@ -30721,7 +30721,7 @@
         <v>3</v>
       </c>
       <c r="B11">
-        <v>101039</v>
+        <v>1010390</v>
       </c>
       <c r="C11" s="10">
         <v>44329</v>

</xml_diff>

<commit_message>
Me queda modificacion aparatado analisis 20-21 y terminar de graficar
</commit_message>
<xml_diff>
--- a/Tabla_Nvasosnuevos.xlsx
+++ b/Tabla_Nvasosnuevos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\minicores\Qca_Bruto\Minicores-Q.canariensis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41092F9C-7644-498C-ACDE-0C9322140032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F210CE60-DF6F-4166-A691-2275F0FB8207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-705" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="newvess" sheetId="1" r:id="rId1"/>
@@ -1519,7 +1519,7 @@
         <v>2</v>
       </c>
       <c r="L27" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -1557,7 +1557,7 @@
         <v>2</v>
       </c>
       <c r="L28" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -1595,7 +1595,7 @@
         <v>2</v>
       </c>
       <c r="L29" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -1633,7 +1633,7 @@
         <v>2</v>
       </c>
       <c r="L30" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -1671,7 +1671,7 @@
         <v>2</v>
       </c>
       <c r="L31" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -1709,7 +1709,7 @@
         <v>2</v>
       </c>
       <c r="L32" s="4">
-        <v>44542</v>
+        <v>44546</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -6193,7 +6193,7 @@
         <v>5</v>
       </c>
       <c r="L150" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
@@ -6231,7 +6231,7 @@
         <v>5</v>
       </c>
       <c r="L151" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
@@ -6269,7 +6269,7 @@
         <v>5</v>
       </c>
       <c r="L152" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
@@ -6307,7 +6307,7 @@
         <v>5</v>
       </c>
       <c r="L153" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
@@ -6345,7 +6345,7 @@
         <v>5</v>
       </c>
       <c r="L154" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
@@ -6383,7 +6383,7 @@
         <v>5</v>
       </c>
       <c r="L155" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
@@ -6421,7 +6421,7 @@
         <v>5</v>
       </c>
       <c r="L156" s="11">
-        <v>44490</v>
+        <v>44483</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
@@ -6611,7 +6611,7 @@
         <v>8</v>
       </c>
       <c r="L161" s="11">
-        <v>44287</v>
+        <v>44315</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
@@ -6649,7 +6649,7 @@
         <v>8</v>
       </c>
       <c r="L162" s="11">
-        <v>44287</v>
+        <v>44315</v>
       </c>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
@@ -6687,7 +6687,7 @@
         <v>8</v>
       </c>
       <c r="L163" s="11">
-        <v>44287</v>
+        <v>44315</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
@@ -30625,7 +30625,7 @@
         <v>760000</v>
       </c>
       <c r="C2" s="10">
-        <v>44329</v>
+        <v>44301</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -30636,7 +30636,7 @@
         <v>160000</v>
       </c>
       <c r="C3" s="10">
-        <v>44343</v>
+        <v>44329</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -30691,7 +30691,7 @@
         <v>56400</v>
       </c>
       <c r="C8" s="10">
-        <v>44215</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -30699,7 +30699,7 @@
         <v>3</v>
       </c>
       <c r="B9">
-        <v>2870000</v>
+        <v>287000</v>
       </c>
       <c r="C9" s="10">
         <v>44287</v>
@@ -30779,7 +30779,7 @@
         <v>96112.072</v>
       </c>
       <c r="C16" s="10">
-        <v>44571</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>